<commit_message>
feat: sludi client rejection reasons
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/reason_list.xlsx
+++ b/mosip_master/xlsx/reason_list.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="120">
   <si>
     <t>lang_code</t>
   </si>
@@ -55,42 +55,48 @@
     <t>CLR</t>
   </si>
   <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>GPM</t>
+  </si>
+  <si>
+    <t>Gender-Photo Mismatch</t>
+  </si>
+  <si>
+    <t>Gender-Photo Mismatch between Gender and Photo</t>
+  </si>
+  <si>
+    <t>IAD</t>
+  </si>
+  <si>
+    <t>Invalid Address</t>
+  </si>
+  <si>
+    <t>Invalid Address found</t>
+  </si>
+  <si>
+    <t>DPG</t>
+  </si>
+  <si>
+    <t>Duplicate Registration</t>
+  </si>
+  <si>
+    <t>Duplicate Registration found</t>
+  </si>
+  <si>
+    <t>OTH</t>
+  </si>
+  <si>
+    <t>Other (specify reason)</t>
+  </si>
+  <si>
+    <t>Any other reason; the supervisor types it in</t>
+  </si>
+  <si>
     <t>TRUE</t>
   </si>
   <si>
-    <t>GPM</t>
-  </si>
-  <si>
-    <t>Gender-Photo Mismatch</t>
-  </si>
-  <si>
-    <t>Gender-Photo Mismatch between Gender and Photo</t>
-  </si>
-  <si>
-    <t>IAD</t>
-  </si>
-  <si>
-    <t>Invalid Address</t>
-  </si>
-  <si>
-    <t>Invalid Address found</t>
-  </si>
-  <si>
-    <t>DPG</t>
-  </si>
-  <si>
-    <t>Duplicate Registration</t>
-  </si>
-  <si>
-    <t>Duplicate Registration found</t>
-  </si>
-  <si>
-    <t>OTH</t>
-  </si>
-  <si>
-    <t>Others</t>
-  </si>
-  <si>
     <t>ADM</t>
   </si>
   <si>
@@ -145,7 +151,10 @@
     <t>நகல் பதிவு கண்டறியப்பட்டது</t>
   </si>
   <si>
-    <t>மற்றவைகள்</t>
+    <t>மற்றவை (காரணத்தைக் குறிப்பிடவும்)</t>
+  </si>
+  <si>
+    <t>வேறு ஏதேனும் காரணம்; மேற்பார்வையாளர் அதைத் தட்டச்சு செய்வார்</t>
   </si>
   <si>
     <t>அனைத்து விவரங்களும் பொருந்துகின்றன</t>
@@ -187,7 +196,10 @@
     <t>අනුපිටපත් ලියාපදිංචියක් හමු විය</t>
   </si>
   <si>
-    <t>වෙනත්</t>
+    <t>වෙනත් (හේතුව සඳහන් කරන්න)</t>
+  </si>
+  <si>
+    <t>වෙනත් ඕනෑම හේතුවක්; අධීක්ෂකවරයා එය ටයිප් කරයි</t>
   </si>
   <si>
     <t>සියලු විස්තර ගැළපේ</t>
@@ -200,6 +212,174 @@
   </si>
   <si>
     <t>සමහර ජනගහන විස්තර ගැළපේ</t>
+  </si>
+  <si>
+    <t>PHM</t>
+  </si>
+  <si>
+    <t>Photo mismatch</t>
+  </si>
+  <si>
+    <t>Captured photo looks inconsistent with the applicant's recorded details (e.g. apparent age far from DOB) or with photos on their supporting documents</t>
+  </si>
+  <si>
+    <t>PHQ</t>
+  </si>
+  <si>
+    <t>Poor photo quality</t>
+  </si>
+  <si>
+    <t>Blurry, bad lighting, face hidden, or doesn't meet ICAO photo rules</t>
+  </si>
+  <si>
+    <t>BIQ</t>
+  </si>
+  <si>
+    <t>Biometric quality issue</t>
+  </si>
+  <si>
+    <t>Fingerprint or iris captures below the quality threshold</t>
+  </si>
+  <si>
+    <t>BEX</t>
+  </si>
+  <si>
+    <t>Biometric exception not justified</t>
+  </si>
+  <si>
+    <t>A missing finger or eye was marked as an exception without proof</t>
+  </si>
+  <si>
+    <t>DDM</t>
+  </si>
+  <si>
+    <t>Demographic details mismatch</t>
+  </si>
+  <si>
+    <t>Name, DOB or address differs from the birth certificate or NIC</t>
+  </si>
+  <si>
+    <t>MSD</t>
+  </si>
+  <si>
+    <t>Missing supporting document</t>
+  </si>
+  <si>
+    <t>A required document wasn't scanned or attached</t>
+  </si>
+  <si>
+    <t>IVD</t>
+  </si>
+  <si>
+    <t>Invalid or unreadable document</t>
+  </si>
+  <si>
+    <t>Expired, damaged, illegible or not an accepted type</t>
+  </si>
+  <si>
+    <t>DUP</t>
+  </si>
+  <si>
+    <t>Suspected duplicate or fraud</t>
+  </si>
+  <si>
+    <t>Identity looks already enrolled, or documents look tampered with</t>
+  </si>
+  <si>
+    <t>ඡායාරූප නොගැළපීම</t>
+  </si>
+  <si>
+    <t>ගත් ඡායාරූපය අයදුම්කරුගේ වාර්තාගත විස්තර (උදා. උපන් දිනයට වඩා බෙහෙවින් වෙනස් පෙනෙන වයස) හෝ සහාය ලේඛනවල ඡායාරූප සමඟ නොගැළපේ</t>
+  </si>
+  <si>
+    <t>දුර්වල ඡායාරූප ගුණාත්මකභාවය</t>
+  </si>
+  <si>
+    <t>බොඳ වූ, ආලෝකය දුර්වල, මුහුණ වැසී ඇති, හෝ ICAO ඡායාරූප නීතිවලට අනුකූල නොවන</t>
+  </si>
+  <si>
+    <t>ජෛවමිතික ගුණාත්මක ගැටලුව</t>
+  </si>
+  <si>
+    <t>ඇඟිලි සලකුණු හෝ අයිරිස් ග්‍රහණය ගුණාත්මක සීමාවට වඩා අඩුය</t>
+  </si>
+  <si>
+    <t>සාධාරණීකරණය නොකළ ජෛවමිතික ව්‍යතිරේකය</t>
+  </si>
+  <si>
+    <t>සාක්ෂි නොමැතිව නැති ඇඟිල්ලක් හෝ ඇසක් ව්‍යතිරේකයක් ලෙස සලකුණු කර ඇත</t>
+  </si>
+  <si>
+    <t>ජනවිකාස විස්තර නොගැළපීම</t>
+  </si>
+  <si>
+    <t>නම, උපන් දිනය හෝ ලිපිනය උප්පැන්න සහතිකයෙන් හෝ ජාතික හැඳුනුම්පතෙන් වෙනස් වේ</t>
+  </si>
+  <si>
+    <t>සහාය ලේඛනය නොමැත</t>
+  </si>
+  <si>
+    <t>අවශ්‍ය ලේඛනයක් ස්කෑන් කර හෝ අමුණා නැත</t>
+  </si>
+  <si>
+    <t>අවලංගු හෝ කියවිය නොහැකි ලේඛනය</t>
+  </si>
+  <si>
+    <t>කල් ඉකුත් වූ, හානි වූ, කියවිය නොහැකි හෝ පිළිගත් වර්ගයක් නොවන</t>
+  </si>
+  <si>
+    <t>සැක සහිත අනුපිටපතක් හෝ වංචාවක්</t>
+  </si>
+  <si>
+    <t>අනන්‍යතාවය දැනටමත් ලියාපදිංචි වී ඇති බව හෝ ලේඛන විකෘති කර ඇති බව පෙනේ</t>
+  </si>
+  <si>
+    <t>புகைப்படம் பொருந்தவில்லை</t>
+  </si>
+  <si>
+    <t>எடுக்கப்பட்ட புகைப்படம் விண்ணப்பதாரரின் பதிவு விவரங்களுடன் (எ.கா. பிறந்த தேதியிலிருந்து மிகவும் வேறுபட்ட தோற்ற வயது) அல்லது ஆதார ஆவணங்களிலுள்ள புகைப்படங்களுடன் பொருந்தவில்லை</t>
+  </si>
+  <si>
+    <t>புகைப்படத்தின் தரம் குறைவு</t>
+  </si>
+  <si>
+    <t>மங்கலானது, போதிய வெளிச்சமின்மை, முகம் மறைக்கப்பட்டுள்ளது அல்லது ICAO புகைப்பட விதிகளுக்கு இணங்கவில்லை</t>
+  </si>
+  <si>
+    <t>உயிரியளவு தரச் சிக்கல்</t>
+  </si>
+  <si>
+    <t>கைரேகை அல்லது கருவிழி பதிவுகள் தர வரம்பிற்குக் கீழே உள்ளன</t>
+  </si>
+  <si>
+    <t>நியாயப்படுத்தப்படாத உயிரியளவு விதிவிலக்கு</t>
+  </si>
+  <si>
+    <t>ஆதாரம் இல்லாமல் இல்லாத விரல் அல்லது கண் விதிவிலக்காகக் குறிக்கப்பட்டுள்ளது</t>
+  </si>
+  <si>
+    <t>மக்கள்தொகை விவரங்கள் பொருந்தவில்லை</t>
+  </si>
+  <si>
+    <t>பெயர், பிறந்த தேதி அல்லது முகவரி பிறப்புச் சான்றிதழ் அல்லது தேசிய அடையாள அட்டையிலிருந்து வேறுபடுகிறது</t>
+  </si>
+  <si>
+    <t>ஆதார ஆவணம் இல்லை</t>
+  </si>
+  <si>
+    <t>தேவையான ஆவணம் ஸ்கேன் செய்யப்படவில்லை அல்லது இணைக்கப்படவில்லை</t>
+  </si>
+  <si>
+    <t>செல்லாத அல்லது படிக்க முடியாத ஆவணம்</t>
+  </si>
+  <si>
+    <t>காலாவதியானது, சேதமடைந்தது, படிக்க முடியாதது அல்லது ஏற்றுக்கொள்ளப்பட்ட வகை அல்ல</t>
+  </si>
+  <si>
+    <t>சந்தேகத்திற்குரிய நகல் அல்லது மோசடி</t>
+  </si>
+  <si>
+    <t>அடையாளம் ஏற்கனவே பதிவுசெய்யப்பட்டதாக அல்லது ஆவணங்கள் சேதப்படுத்தப்பட்டதாகத் தெரிகிறது</t>
   </si>
 </sst>
 </file>
@@ -562,14 +742,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="70.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="93.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -589,7 +769,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -609,7 +789,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -629,7 +809,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -649,7 +829,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -669,7 +849,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -680,107 +860,107 @@
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" t="s">
         <v>27</v>
       </c>
-      <c r="D8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" t="s">
-        <v>25</v>
-      </c>
       <c r="F8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -789,18 +969,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -809,18 +989,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -829,18 +1009,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B14" t="s">
         <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -849,118 +1029,118 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
         <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D15" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" t="s">
         <v>32</v>
       </c>
-      <c r="B16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" t="s">
-        <v>43</v>
-      </c>
-      <c r="D17" t="s">
-        <v>43</v>
-      </c>
-      <c r="E17" t="s">
-        <v>25</v>
-      </c>
-      <c r="F17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" t="s">
-        <v>25</v>
-      </c>
-      <c r="F18" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" t="s">
-        <v>30</v>
-      </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E19" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F19" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B20" t="s">
         <v>7</v>
       </c>
       <c r="C20" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -969,18 +1149,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -989,18 +1169,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B22" t="s">
         <v>15</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D22" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1009,18 +1189,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s">
         <v>18</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1029,104 +1209,584 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
         <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D24" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D25" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E25" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F25" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E26" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F26" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C27" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D27" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E27" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F27" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D28" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E28" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F28" t="s">
-        <v>11</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" t="s">
+        <v>68</v>
+      </c>
+      <c r="D30" t="s">
+        <v>69</v>
+      </c>
+      <c r="E30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" t="s">
+        <v>71</v>
+      </c>
+      <c r="D31" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" t="s">
+        <v>74</v>
+      </c>
+      <c r="D32" t="s">
+        <v>75</v>
+      </c>
+      <c r="E32" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>6</v>
+      </c>
+      <c r="B33" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" t="s">
+        <v>77</v>
+      </c>
+      <c r="D33" t="s">
+        <v>78</v>
+      </c>
+      <c r="E33" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" t="s">
+        <v>81</v>
+      </c>
+      <c r="E34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" t="s">
+        <v>84</v>
+      </c>
+      <c r="E35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>6</v>
+      </c>
+      <c r="B36" t="s">
+        <v>85</v>
+      </c>
+      <c r="C36" t="s">
+        <v>86</v>
+      </c>
+      <c r="D36" t="s">
+        <v>87</v>
+      </c>
+      <c r="E36" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" t="s">
+        <v>88</v>
+      </c>
+      <c r="D37" t="s">
+        <v>89</v>
+      </c>
+      <c r="E37" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38" t="s">
+        <v>90</v>
+      </c>
+      <c r="D38" t="s">
+        <v>91</v>
+      </c>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>49</v>
+      </c>
+      <c r="B39" t="s">
+        <v>70</v>
+      </c>
+      <c r="C39" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39" t="s">
+        <v>93</v>
+      </c>
+      <c r="E39" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" t="s">
+        <v>94</v>
+      </c>
+      <c r="D40" t="s">
+        <v>95</v>
+      </c>
+      <c r="E40" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" t="s">
+        <v>49</v>
+      </c>
+      <c r="B41" t="s">
+        <v>76</v>
+      </c>
+      <c r="C41" t="s">
+        <v>96</v>
+      </c>
+      <c r="D41" t="s">
+        <v>97</v>
+      </c>
+      <c r="E41" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42" t="s">
+        <v>79</v>
+      </c>
+      <c r="C42" t="s">
+        <v>98</v>
+      </c>
+      <c r="D42" t="s">
+        <v>99</v>
+      </c>
+      <c r="E42" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" t="s">
+        <v>100</v>
+      </c>
+      <c r="D43" t="s">
+        <v>101</v>
+      </c>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" t="s">
+        <v>49</v>
+      </c>
+      <c r="B44" t="s">
+        <v>85</v>
+      </c>
+      <c r="C44" t="s">
+        <v>102</v>
+      </c>
+      <c r="D44" t="s">
+        <v>103</v>
+      </c>
+      <c r="E44" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" t="s">
+        <v>34</v>
+      </c>
+      <c r="B45" t="s">
+        <v>64</v>
+      </c>
+      <c r="C45" t="s">
+        <v>104</v>
+      </c>
+      <c r="D45" t="s">
+        <v>105</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" t="s">
+        <v>34</v>
+      </c>
+      <c r="B46" t="s">
+        <v>67</v>
+      </c>
+      <c r="C46" t="s">
+        <v>106</v>
+      </c>
+      <c r="D46" t="s">
+        <v>107</v>
+      </c>
+      <c r="E46" t="s">
+        <v>10</v>
+      </c>
+      <c r="F46" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" t="s">
+        <v>34</v>
+      </c>
+      <c r="B47" t="s">
+        <v>70</v>
+      </c>
+      <c r="C47" t="s">
+        <v>108</v>
+      </c>
+      <c r="D47" t="s">
+        <v>109</v>
+      </c>
+      <c r="E47" t="s">
+        <v>10</v>
+      </c>
+      <c r="F47" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" t="s">
+        <v>34</v>
+      </c>
+      <c r="B48" t="s">
+        <v>73</v>
+      </c>
+      <c r="C48" t="s">
+        <v>110</v>
+      </c>
+      <c r="D48" t="s">
+        <v>111</v>
+      </c>
+      <c r="E48" t="s">
+        <v>10</v>
+      </c>
+      <c r="F48" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" t="s">
+        <v>34</v>
+      </c>
+      <c r="B49" t="s">
+        <v>76</v>
+      </c>
+      <c r="C49" t="s">
+        <v>112</v>
+      </c>
+      <c r="D49" t="s">
+        <v>113</v>
+      </c>
+      <c r="E49" t="s">
+        <v>10</v>
+      </c>
+      <c r="F49" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" t="s">
+        <v>34</v>
+      </c>
+      <c r="B50" t="s">
+        <v>79</v>
+      </c>
+      <c r="C50" t="s">
+        <v>114</v>
+      </c>
+      <c r="D50" t="s">
+        <v>115</v>
+      </c>
+      <c r="E50" t="s">
+        <v>10</v>
+      </c>
+      <c r="F50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" t="s">
+        <v>34</v>
+      </c>
+      <c r="B51" t="s">
+        <v>82</v>
+      </c>
+      <c r="C51" t="s">
+        <v>116</v>
+      </c>
+      <c r="D51" t="s">
+        <v>117</v>
+      </c>
+      <c r="E51" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" t="s">
+        <v>34</v>
+      </c>
+      <c r="B52" t="s">
+        <v>85</v>
+      </c>
+      <c r="C52" t="s">
+        <v>118</v>
+      </c>
+      <c r="D52" t="s">
+        <v>119</v>
+      </c>
+      <c r="E52" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>